<commit_message>
Ajout fiche de mission E5 (Documents + Entreprise) et tableau de synthese mis a jour
</commit_message>
<xml_diff>
--- a/assets/BTS_SIO_Annexe_6_Epreuve E5 - Tableau de synthese_2026.xlsx
+++ b/assets/BTS_SIO_Annexe_6_Epreuve E5 - Tableau de synthese_2026.xlsx
@@ -1262,7 +1262,7 @@
     <row r="5" ht="39.95" customHeight="1" thickBot="1">
       <c r="A5" s="56" t="inlineStr">
         <is>
-          <t>Adresse URL du portfolio : https://sahed-portfolio.pages.dev/</t>
+          <t>Adresse URL du portfolio : https://portfolio-v2-ev1.pages.dev</t>
         </is>
       </c>
       <c r="B5" s="57" t="n"/>
@@ -1469,14 +1469,34 @@
       <c r="H11" s="22" t="n"/>
     </row>
     <row r="12" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A12" s="13" t="n"/>
-      <c r="B12" s="11" t="n"/>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Portfolio professionnel en ligne, sécurisé « secure by design » — conception et mise en ligne du portfolio (hébergement serverless, API de contact, en-têtes de sécurité HTTP), veille technologique et formalisation du projet professionnel (documents : site en ligne, dépôt Git)</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>2026 (en continu)</t>
+        </is>
+      </c>
       <c r="C12" s="21" t="n"/>
       <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G12" s="21" t="n"/>
-      <c r="H12" s="22" t="n"/>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A13" s="13" t="n"/>
@@ -1555,12 +1575,12 @@
     <row r="20" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Modernisation du déploiement d'environnements de test et renforcement de la sécurité des accès aux outils internes — conteneurisation Docker/Kubernetes, authentification par token, gestion des droits RBAC, pipelines CI/CD GitHub Actions (documents : pipeline CI/CD, configuration RBAC)</t>
+          <t>Fiabilisation et mise à disposition d'une plateforme interne de laboratoires de cybersécurité — test, diagnostic et réparation de 26 images de conteneurs Docker (SIEM, pfSense, Kali, OSINT, cryptographie), validation (construction, exécution, déploiement Kubernetes) et livraison pour publication (documents : procédure de test, guide de dépannage, dépôt Git)</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Juin - Juillet 2026 (8 semaines, dates exactes à confirmer)</t>
+          <t>Juin – Juillet 2026 (dates exactes à confirmer)</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
@@ -1589,30 +1609,22 @@
     <row r="21" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Développement d'évolutions fonctionnelles sur le SIS interne MyCaplogySchool (FlexCampus) — module présence/absences et justificatifs, évaluations (barèmes, bulletins), sécurisation et accessibilité des profils élève/professeur (documents : dépôt Git, spécifications fonctionnelles)</t>
+          <t>Mise en service et supervision de laboratoires SIEM (Wazuh, Splunk, ELK) — déploiement sur Kubernetes, validation de la détection (surveillance d'intégrité de fichiers) et de l'authentification des outils (documents : captures de supervision, journaux de détection)</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Juin - Juillet 2026 (8 semaines, dates exactes à confirmer)</t>
-        </is>
-      </c>
-      <c r="C21" s="21" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Juin – Juillet 2026 (dates exactes à confirmer)</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="n"/>
       <c r="D21" s="21" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
       <c r="E21" s="21" t="n"/>
-      <c r="F21" s="21" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F21" s="21" t="n"/>
       <c r="G21" s="21" t="inlineStr">
         <is>
           <t>X</t>
@@ -1621,12 +1633,32 @@
       <c r="H21" s="22" t="n"/>
     </row>
     <row r="22" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A22" s="13" t="n"/>
-      <c r="B22" s="11" t="n"/>
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Audit de sécurité et évolutions d'une application web interne de gestion — revue de code (OWASP), correction d'une faille de contrôle d'accès (IDOR), gestion des droits (RBAC) et déploiement automatisé (CI/CD), documentation de passation (documents : rapport d'audit, dépôt Git)</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Juin – Juillet 2026 (dates exactes à confirmer)</t>
+        </is>
+      </c>
       <c r="C22" s="21" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="21" t="n"/>
-      <c r="F22" s="21" t="n"/>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G22" s="21" t="n"/>
       <c r="H22" s="22" t="n"/>
     </row>

</xml_diff>